<commit_message>
Added Forward_Barcode and Reverse_Barcode to field list.
</commit_message>
<xml_diff>
--- a/README/igseq_database_fields.xlsx
+++ b/README/igseq_database_fields.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="25516"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="27907"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chrisfucile/Repos/IgSeq/README/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="64060" yWindow="-14180" windowWidth="27140" windowHeight="23560" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="11260" yWindow="460" windowWidth="27140" windowHeight="22680" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="140000" refMode="R1C1" concurrentCalc="0"/>
+  <calcPr calcId="150001" refMode="R1C1" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr defaultImageDpi="32767"/>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -20,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="334">
   <si>
     <t>LineageID</t>
   </si>
@@ -1013,6 +1021,15 @@
   </si>
   <si>
     <t>undef</t>
+  </si>
+  <si>
+    <t>Forward_Barcode</t>
+  </si>
+  <si>
+    <t>Reverse_Barcode</t>
+  </si>
+  <si>
+    <t>TEXT</t>
   </si>
 </sst>
 </file>
@@ -1183,6 +1200,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1509,7 +1531,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D167"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.33203125" bestFit="1" customWidth="1"/>
@@ -1517,7 +1539,7 @@
     <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>319</v>
       </c>
@@ -1531,7 +1553,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1545,7 +1567,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1559,7 +1581,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1573,7 +1595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
         <v>163</v>
       </c>
@@ -1581,7 +1603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>323</v>
       </c>
@@ -1589,7 +1611,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>324</v>
       </c>
@@ -1597,7 +1619,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4</v>
       </c>
@@ -1605,7 +1627,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>5</v>
       </c>
@@ -1619,7 +1641,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>6</v>
       </c>
@@ -1633,7 +1655,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>7</v>
       </c>
@@ -1647,7 +1669,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
         <v>314</v>
       </c>
@@ -1655,7 +1677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
         <v>316</v>
       </c>
@@ -1663,7 +1685,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
         <v>317</v>
       </c>
@@ -1671,7 +1693,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>8</v>
       </c>
@@ -1685,7 +1707,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>9</v>
       </c>
@@ -1699,7 +1721,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>10</v>
       </c>
@@ -1713,7 +1735,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>11</v>
       </c>
@@ -1727,7 +1749,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>12</v>
       </c>
@@ -1741,7 +1763,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>13</v>
       </c>
@@ -1755,7 +1777,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>14</v>
       </c>
@@ -1769,7 +1791,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>15</v>
       </c>
@@ -1783,7 +1805,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>16</v>
       </c>
@@ -1797,7 +1819,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>17</v>
       </c>
@@ -1811,7 +1833,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>18</v>
       </c>
@@ -1825,7 +1847,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>19</v>
       </c>
@@ -1839,7 +1861,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>20</v>
       </c>
@@ -1847,7 +1869,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>21</v>
       </c>
@@ -1861,7 +1883,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>22</v>
       </c>
@@ -1875,7 +1897,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>23</v>
       </c>
@@ -1889,7 +1911,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>24</v>
       </c>
@@ -1903,7 +1925,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>25</v>
       </c>
@@ -1917,7 +1939,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>26</v>
       </c>
@@ -1931,7 +1953,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>27</v>
       </c>
@@ -1945,7 +1967,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>28</v>
       </c>
@@ -1959,7 +1981,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>29</v>
       </c>
@@ -1973,7 +1995,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>30</v>
       </c>
@@ -1987,7 +2009,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>31</v>
       </c>
@@ -2001,7 +2023,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>32</v>
       </c>
@@ -2015,7 +2037,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>33</v>
       </c>
@@ -2023,7 +2045,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>34</v>
       </c>
@@ -2037,7 +2059,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>35</v>
       </c>
@@ -2051,7 +2073,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>36</v>
       </c>
@@ -2065,7 +2087,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>37</v>
       </c>
@@ -2079,7 +2101,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>38</v>
       </c>
@@ -2093,7 +2115,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>39</v>
       </c>
@@ -2107,7 +2129,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>40</v>
       </c>
@@ -2121,7 +2143,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>41</v>
       </c>
@@ -2135,7 +2157,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>42</v>
       </c>
@@ -2149,7 +2171,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>43</v>
       </c>
@@ -2163,7 +2185,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>44</v>
       </c>
@@ -2177,7 +2199,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>45</v>
       </c>
@@ -2191,7 +2213,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>46</v>
       </c>
@@ -2205,7 +2227,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>47</v>
       </c>
@@ -2219,7 +2241,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>48</v>
       </c>
@@ -2233,7 +2255,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>49</v>
       </c>
@@ -2247,7 +2269,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>50</v>
       </c>
@@ -2261,7 +2283,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>51</v>
       </c>
@@ -2275,7 +2297,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>52</v>
       </c>
@@ -2289,7 +2311,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>53</v>
       </c>
@@ -2303,7 +2325,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>54</v>
       </c>
@@ -2317,7 +2339,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>55</v>
       </c>
@@ -2331,7 +2353,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>56</v>
       </c>
@@ -2345,7 +2367,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>57</v>
       </c>
@@ -2359,7 +2381,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>58</v>
       </c>
@@ -2373,7 +2395,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>59</v>
       </c>
@@ -2387,7 +2409,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>60</v>
       </c>
@@ -2401,7 +2423,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>61</v>
       </c>
@@ -2415,7 +2437,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>62</v>
       </c>
@@ -2429,7 +2451,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="70" spans="1:4">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>63</v>
       </c>
@@ -2443,7 +2465,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>64</v>
       </c>
@@ -2457,7 +2479,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>65</v>
       </c>
@@ -2471,7 +2493,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>66</v>
       </c>
@@ -2485,7 +2507,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>67</v>
       </c>
@@ -2499,7 +2521,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>68</v>
       </c>
@@ -2513,7 +2535,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>69</v>
       </c>
@@ -2527,7 +2549,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>70</v>
       </c>
@@ -2541,7 +2563,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>71</v>
       </c>
@@ -2555,7 +2577,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="79" spans="1:4">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>72</v>
       </c>
@@ -2569,7 +2591,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="80" spans="1:4">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>73</v>
       </c>
@@ -2583,7 +2605,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>74</v>
       </c>
@@ -2597,7 +2619,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>75</v>
       </c>
@@ -2611,7 +2633,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>76</v>
       </c>
@@ -2625,7 +2647,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>77</v>
       </c>
@@ -2639,7 +2661,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>78</v>
       </c>
@@ -2653,7 +2675,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>79</v>
       </c>
@@ -2667,7 +2689,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>80</v>
       </c>
@@ -2681,7 +2703,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="88" spans="1:4">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>81</v>
       </c>
@@ -2695,7 +2717,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="89" spans="1:4">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>82</v>
       </c>
@@ -2709,7 +2731,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="90" spans="1:4">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>83</v>
       </c>
@@ -2723,7 +2745,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="91" spans="1:4">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>84</v>
       </c>
@@ -2737,7 +2759,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="92" spans="1:4">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>85</v>
       </c>
@@ -2751,7 +2773,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="93" spans="1:4">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>86</v>
       </c>
@@ -2765,7 +2787,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="94" spans="1:4">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>87</v>
       </c>
@@ -2779,7 +2801,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="95" spans="1:4">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>88</v>
       </c>
@@ -2793,7 +2815,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="96" spans="1:4">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>89</v>
       </c>
@@ -2807,7 +2829,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="97" spans="1:4">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>90</v>
       </c>
@@ -2821,7 +2843,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="98" spans="1:4">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>91</v>
       </c>
@@ -2835,7 +2857,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="99" spans="1:4">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>92</v>
       </c>
@@ -2849,7 +2871,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="100" spans="1:4">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>93</v>
       </c>
@@ -2863,7 +2885,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="101" spans="1:4">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>94</v>
       </c>
@@ -2877,7 +2899,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="102" spans="1:4">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>95</v>
       </c>
@@ -2891,7 +2913,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="103" spans="1:4">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>96</v>
       </c>
@@ -2905,7 +2927,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="104" spans="1:4">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>97</v>
       </c>
@@ -2919,7 +2941,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="105" spans="1:4">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>98</v>
       </c>
@@ -2933,7 +2955,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="106" spans="1:4">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>99</v>
       </c>
@@ -2947,7 +2969,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="107" spans="1:4">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>100</v>
       </c>
@@ -2961,7 +2983,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="108" spans="1:4">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>101</v>
       </c>
@@ -2975,7 +2997,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="109" spans="1:4">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>102</v>
       </c>
@@ -2989,7 +3011,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="110" spans="1:4">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>103</v>
       </c>
@@ -3003,7 +3025,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="111" spans="1:4">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>104</v>
       </c>
@@ -3017,7 +3039,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="112" spans="1:4">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>105</v>
       </c>
@@ -3031,7 +3053,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="113" spans="1:4">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>106</v>
       </c>
@@ -3045,7 +3067,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="114" spans="1:4">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>107</v>
       </c>
@@ -3059,7 +3081,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="115" spans="1:4">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>108</v>
       </c>
@@ -3073,7 +3095,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="116" spans="1:4">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>109</v>
       </c>
@@ -3087,7 +3109,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="117" spans="1:4">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>110</v>
       </c>
@@ -3101,7 +3123,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="118" spans="1:4">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>111</v>
       </c>
@@ -3115,7 +3137,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="119" spans="1:4">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>112</v>
       </c>
@@ -3129,7 +3151,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="120" spans="1:4">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>113</v>
       </c>
@@ -3143,7 +3165,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="121" spans="1:4">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>114</v>
       </c>
@@ -3157,7 +3179,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="122" spans="1:4">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>115</v>
       </c>
@@ -3171,7 +3193,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="123" spans="1:4">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>116</v>
       </c>
@@ -3185,7 +3207,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="124" spans="1:4">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>117</v>
       </c>
@@ -3199,7 +3221,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="125" spans="1:4">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>118</v>
       </c>
@@ -3213,7 +3235,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="126" spans="1:4">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>119</v>
       </c>
@@ -3227,7 +3249,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="127" spans="1:4">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>120</v>
       </c>
@@ -3241,7 +3263,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="128" spans="1:4">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>121</v>
       </c>
@@ -3255,7 +3277,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="129" spans="1:4">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>122</v>
       </c>
@@ -3269,7 +3291,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="130" spans="1:4">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>123</v>
       </c>
@@ -3283,7 +3305,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="131" spans="1:4">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>124</v>
       </c>
@@ -3297,7 +3319,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="132" spans="1:4">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>125</v>
       </c>
@@ -3311,7 +3333,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="133" spans="1:4">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>126</v>
       </c>
@@ -3325,7 +3347,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="134" spans="1:4">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>127</v>
       </c>
@@ -3339,7 +3361,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="135" spans="1:4">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>128</v>
       </c>
@@ -3353,7 +3375,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="136" spans="1:4">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>129</v>
       </c>
@@ -3367,7 +3389,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="137" spans="1:4">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>130</v>
       </c>
@@ -3381,7 +3403,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="138" spans="1:4">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>131</v>
       </c>
@@ -3395,7 +3417,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="139" spans="1:4">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>132</v>
       </c>
@@ -3409,7 +3431,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="140" spans="1:4">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>133</v>
       </c>
@@ -3423,7 +3445,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="141" spans="1:4">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>134</v>
       </c>
@@ -3437,7 +3459,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="142" spans="1:4">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>135</v>
       </c>
@@ -3451,7 +3473,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="143" spans="1:4">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>136</v>
       </c>
@@ -3465,7 +3487,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="144" spans="1:4">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>137</v>
       </c>
@@ -3479,7 +3501,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="145" spans="1:4">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>138</v>
       </c>
@@ -3493,7 +3515,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="146" spans="1:4">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>139</v>
       </c>
@@ -3507,7 +3529,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="147" spans="1:4">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>140</v>
       </c>
@@ -3521,7 +3543,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="148" spans="1:4">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>141</v>
       </c>
@@ -3535,7 +3557,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="149" spans="1:4">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>142</v>
       </c>
@@ -3549,7 +3571,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="150" spans="1:4">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>143</v>
       </c>
@@ -3563,7 +3585,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="151" spans="1:4">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>144</v>
       </c>
@@ -3577,7 +3599,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="152" spans="1:4">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>145</v>
       </c>
@@ -3591,7 +3613,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="153" spans="1:4">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>146</v>
       </c>
@@ -3605,7 +3627,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="154" spans="1:4">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>147</v>
       </c>
@@ -3619,7 +3641,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="155" spans="1:4">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>148</v>
       </c>
@@ -3633,7 +3655,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="156" spans="1:4">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>149</v>
       </c>
@@ -3647,7 +3669,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="157" spans="1:4">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>150</v>
       </c>
@@ -3661,7 +3683,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="158" spans="1:4">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>151</v>
       </c>
@@ -3675,7 +3697,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="159" spans="1:4">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>152</v>
       </c>
@@ -3689,7 +3711,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="160" spans="1:4">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>153</v>
       </c>
@@ -3703,7 +3725,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="161" spans="1:4">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>154</v>
       </c>
@@ -3717,7 +3739,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="162" spans="1:4">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>155</v>
       </c>
@@ -3731,7 +3753,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="163" spans="1:4">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>156</v>
       </c>
@@ -3745,7 +3767,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="164" spans="1:4">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>157</v>
       </c>
@@ -3759,7 +3781,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="165" spans="1:4">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>158</v>
       </c>
@@ -3773,7 +3795,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="166" spans="1:4">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>159</v>
       </c>
@@ -3787,7 +3809,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="167" spans="1:4">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>160</v>
       </c>
@@ -3804,18 +3826,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:FG181"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.1640625" bestFit="1" customWidth="1"/>
@@ -3825,7 +3842,7 @@
     <col min="6" max="6" width="18.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>329</v>
       </c>
@@ -3843,7 +3860,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>B2-1</f>
         <v>2</v>
@@ -3861,7 +3878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>330</v>
       </c>
@@ -3872,7 +3889,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>330</v>
       </c>
@@ -3883,7 +3900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>330</v>
       </c>
@@ -3894,7 +3911,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <f>B6-1</f>
         <v>1</v>
@@ -3912,7 +3929,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <f>B7-1</f>
         <v>0</v>
@@ -3930,7 +3947,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <f>B8-1</f>
         <v>4</v>
@@ -3948,7 +3965,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <f>B9-1</f>
         <v>6</v>
@@ -3966,7 +3983,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <f>B10-1</f>
         <v>5</v>
@@ -3984,7 +4001,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" ref="A11:A13" si="0">B11-1</f>
         <v>7</v>
@@ -3999,7 +4016,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -4014,7 +4031,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -4029,9 +4046,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
-        <f>B14-1</f>
+        <f t="shared" ref="A14:A45" si="1">B14-1</f>
         <v>10</v>
       </c>
       <c r="B14">
@@ -4047,9 +4064,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
-        <f>B15-1</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="B15">
@@ -4065,9 +4082,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
-        <f>B16-1</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="B16">
@@ -4083,9 +4100,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
-        <f>B17-1</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="B17">
@@ -4101,9 +4118,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
-        <f>B18-1</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="B18">
@@ -4119,9 +4136,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
-        <f>B19-1</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="B19">
@@ -4137,9 +4154,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
-        <f>B20-1</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="B20">
@@ -4155,9 +4172,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
-        <f>B21-1</f>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="B21">
@@ -4173,9 +4190,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
-        <f>B22-1</f>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="B22">
@@ -4191,9 +4208,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
-        <f>B23-1</f>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="B23">
@@ -4209,9 +4226,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
-        <f>B24-1</f>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="B24">
@@ -4227,9 +4244,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
-        <f>B25-1</f>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="B25">
@@ -4245,9 +4262,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
-        <f>B26-1</f>
+        <f t="shared" si="1"/>
         <v>162</v>
       </c>
       <c r="B26">
@@ -4264,9 +4281,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
-        <f>B27-1</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="B27">
@@ -4282,9 +4299,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
-        <f>B28-1</f>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="B28">
@@ -4300,9 +4317,9 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
-        <f>B29-1</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="B29">
@@ -4318,9 +4335,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30">
-        <f>B30-1</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="B30">
@@ -4336,9 +4353,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31">
-        <f>B31-1</f>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="B31">
@@ -4354,9 +4371,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32">
-        <f>B32-1</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="B32">
@@ -4372,9 +4389,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
-        <f>B33-1</f>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="B33">
@@ -4390,9 +4407,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
-        <f>B34-1</f>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="B34">
@@ -4408,9 +4425,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
-        <f>B35-1</f>
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="B35">
@@ -4426,9 +4443,9 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36">
-        <f>B36-1</f>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="B36">
@@ -4444,9 +4461,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37">
-        <f>B37-1</f>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="B37">
@@ -4462,9 +4479,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38">
-        <f>B38-1</f>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="B38">
@@ -4480,9 +4497,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39">
-        <f>B39-1</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="B39">
@@ -4501,9 +4518,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40">
-        <f>B40-1</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="B40">
@@ -4522,9 +4539,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41">
-        <f>B41-1</f>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="B41">
@@ -4543,9 +4560,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42">
-        <f>B42-1</f>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="B42">
@@ -4564,9 +4581,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
-        <f>B43-1</f>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="B43">
@@ -4585,9 +4602,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
-        <f>B44-1</f>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="B44">
@@ -4606,9 +4623,9 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
-        <f>B45-1</f>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="B45">
@@ -4627,9 +4644,9 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
-        <f>B46-1</f>
+        <f t="shared" ref="A46:A77" si="2">B46-1</f>
         <v>43</v>
       </c>
       <c r="B46">
@@ -4648,9 +4665,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47">
-        <f>B47-1</f>
+        <f t="shared" si="2"/>
         <v>44</v>
       </c>
       <c r="B47">
@@ -4669,9 +4686,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48">
-        <f>B48-1</f>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="B48">
@@ -4690,9 +4707,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49">
-        <f>B49-1</f>
+        <f t="shared" si="2"/>
         <v>46</v>
       </c>
       <c r="B49">
@@ -4711,9 +4728,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50">
-        <f>B50-1</f>
+        <f t="shared" si="2"/>
         <v>47</v>
       </c>
       <c r="B50">
@@ -4732,9 +4749,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51">
-        <f>B51-1</f>
+        <f t="shared" si="2"/>
         <v>48</v>
       </c>
       <c r="B51">
@@ -4753,9 +4770,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52">
-        <f>B52-1</f>
+        <f t="shared" si="2"/>
         <v>49</v>
       </c>
       <c r="B52">
@@ -4774,9 +4791,9 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53">
-        <f>B53-1</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="B53">
@@ -4795,9 +4812,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54">
-        <f>B54-1</f>
+        <f t="shared" si="2"/>
         <v>51</v>
       </c>
       <c r="B54">
@@ -4816,9 +4833,9 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55">
-        <f>B55-1</f>
+        <f t="shared" si="2"/>
         <v>52</v>
       </c>
       <c r="B55">
@@ -4837,9 +4854,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56">
-        <f>B56-1</f>
+        <f t="shared" si="2"/>
         <v>53</v>
       </c>
       <c r="B56">
@@ -4858,9 +4875,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57">
-        <f>B57-1</f>
+        <f t="shared" si="2"/>
         <v>54</v>
       </c>
       <c r="B57">
@@ -4879,9 +4896,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58">
-        <f>B58-1</f>
+        <f t="shared" si="2"/>
         <v>55</v>
       </c>
       <c r="B58">
@@ -4900,9 +4917,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59">
-        <f>B59-1</f>
+        <f t="shared" si="2"/>
         <v>56</v>
       </c>
       <c r="B59">
@@ -4921,9 +4938,9 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60">
-        <f>B60-1</f>
+        <f t="shared" si="2"/>
         <v>57</v>
       </c>
       <c r="B60">
@@ -4942,9 +4959,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61">
-        <f>B61-1</f>
+        <f t="shared" si="2"/>
         <v>58</v>
       </c>
       <c r="B61">
@@ -4963,9 +4980,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62">
-        <f>B62-1</f>
+        <f t="shared" si="2"/>
         <v>59</v>
       </c>
       <c r="B62">
@@ -4984,9 +5001,9 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63">
-        <f>B63-1</f>
+        <f t="shared" si="2"/>
         <v>60</v>
       </c>
       <c r="B63">
@@ -5005,9 +5022,9 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64">
-        <f>B64-1</f>
+        <f t="shared" si="2"/>
         <v>61</v>
       </c>
       <c r="B64">
@@ -5026,9 +5043,9 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65">
-        <f>B65-1</f>
+        <f t="shared" si="2"/>
         <v>62</v>
       </c>
       <c r="B65">
@@ -5047,9 +5064,9 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66">
-        <f>B66-1</f>
+        <f t="shared" si="2"/>
         <v>63</v>
       </c>
       <c r="B66">
@@ -5068,9 +5085,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67">
-        <f>B67-1</f>
+        <f t="shared" si="2"/>
         <v>64</v>
       </c>
       <c r="B67">
@@ -5089,9 +5106,9 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68">
-        <f>B68-1</f>
+        <f t="shared" si="2"/>
         <v>65</v>
       </c>
       <c r="B68">
@@ -5110,9 +5127,9 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69">
-        <f>B69-1</f>
+        <f t="shared" si="2"/>
         <v>66</v>
       </c>
       <c r="B69">
@@ -5131,9 +5148,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70">
-        <f>B70-1</f>
+        <f t="shared" si="2"/>
         <v>67</v>
       </c>
       <c r="B70">
@@ -5152,9 +5169,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71">
-        <f>B71-1</f>
+        <f t="shared" si="2"/>
         <v>68</v>
       </c>
       <c r="B71">
@@ -5173,9 +5190,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72">
-        <f>B72-1</f>
+        <f t="shared" si="2"/>
         <v>69</v>
       </c>
       <c r="B72">
@@ -5194,9 +5211,9 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73">
-        <f>B73-1</f>
+        <f t="shared" si="2"/>
         <v>70</v>
       </c>
       <c r="B73">
@@ -5215,9 +5232,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74">
-        <f>B74-1</f>
+        <f t="shared" si="2"/>
         <v>71</v>
       </c>
       <c r="B74">
@@ -5236,9 +5253,9 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75">
-        <f>B75-1</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="B75">
@@ -5257,9 +5274,9 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76">
-        <f>B76-1</f>
+        <f t="shared" si="2"/>
         <v>73</v>
       </c>
       <c r="B76">
@@ -5278,9 +5295,9 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77">
-        <f>B77-1</f>
+        <f t="shared" si="2"/>
         <v>74</v>
       </c>
       <c r="B77">
@@ -5299,9 +5316,9 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78">
-        <f>B78-1</f>
+        <f t="shared" ref="A78:A109" si="3">B78-1</f>
         <v>75</v>
       </c>
       <c r="B78">
@@ -5320,9 +5337,9 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79">
-        <f>B79-1</f>
+        <f t="shared" si="3"/>
         <v>76</v>
       </c>
       <c r="B79">
@@ -5341,9 +5358,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80">
-        <f>B80-1</f>
+        <f t="shared" si="3"/>
         <v>77</v>
       </c>
       <c r="B80">
@@ -5362,9 +5379,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81">
-        <f>B81-1</f>
+        <f t="shared" si="3"/>
         <v>78</v>
       </c>
       <c r="B81">
@@ -5383,9 +5400,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82">
-        <f>B82-1</f>
+        <f t="shared" si="3"/>
         <v>79</v>
       </c>
       <c r="B82">
@@ -5404,9 +5421,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83">
-        <f>B83-1</f>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="B83">
@@ -5425,9 +5442,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84">
-        <f>B84-1</f>
+        <f t="shared" si="3"/>
         <v>81</v>
       </c>
       <c r="B84">
@@ -5446,9 +5463,9 @@
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85">
-        <f>B85-1</f>
+        <f t="shared" si="3"/>
         <v>82</v>
       </c>
       <c r="B85">
@@ -5467,9 +5484,9 @@
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86">
-        <f>B86-1</f>
+        <f t="shared" si="3"/>
         <v>83</v>
       </c>
       <c r="B86">
@@ -5488,9 +5505,9 @@
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87">
-        <f>B87-1</f>
+        <f t="shared" si="3"/>
         <v>84</v>
       </c>
       <c r="B87">
@@ -5509,9 +5526,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88">
-        <f>B88-1</f>
+        <f t="shared" si="3"/>
         <v>85</v>
       </c>
       <c r="B88">
@@ -5530,9 +5547,9 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89">
-        <f>B89-1</f>
+        <f t="shared" si="3"/>
         <v>86</v>
       </c>
       <c r="B89">
@@ -5551,9 +5568,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90">
-        <f>B90-1</f>
+        <f t="shared" si="3"/>
         <v>87</v>
       </c>
       <c r="B90">
@@ -5572,9 +5589,9 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91">
-        <f>B91-1</f>
+        <f t="shared" si="3"/>
         <v>88</v>
       </c>
       <c r="B91">
@@ -5593,9 +5610,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92">
-        <f>B92-1</f>
+        <f t="shared" si="3"/>
         <v>89</v>
       </c>
       <c r="B92">
@@ -5614,9 +5631,9 @@
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93">
-        <f>B93-1</f>
+        <f t="shared" si="3"/>
         <v>90</v>
       </c>
       <c r="B93">
@@ -5635,9 +5652,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94">
-        <f>B94-1</f>
+        <f t="shared" si="3"/>
         <v>91</v>
       </c>
       <c r="B94">
@@ -5656,9 +5673,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95">
-        <f>B95-1</f>
+        <f t="shared" si="3"/>
         <v>92</v>
       </c>
       <c r="B95">
@@ -5677,9 +5694,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96">
-        <f>B96-1</f>
+        <f t="shared" si="3"/>
         <v>93</v>
       </c>
       <c r="B96">
@@ -5698,9 +5715,9 @@
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97">
-        <f>B97-1</f>
+        <f t="shared" si="3"/>
         <v>94</v>
       </c>
       <c r="B97">
@@ -5719,9 +5736,9 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98">
-        <f>B98-1</f>
+        <f t="shared" si="3"/>
         <v>95</v>
       </c>
       <c r="B98">
@@ -5740,9 +5757,9 @@
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99">
-        <f>B99-1</f>
+        <f t="shared" si="3"/>
         <v>96</v>
       </c>
       <c r="B99">
@@ -5761,9 +5778,9 @@
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100">
-        <f>B100-1</f>
+        <f t="shared" si="3"/>
         <v>97</v>
       </c>
       <c r="B100">
@@ -5782,9 +5799,9 @@
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101">
-        <f>B101-1</f>
+        <f t="shared" si="3"/>
         <v>98</v>
       </c>
       <c r="B101">
@@ -5803,9 +5820,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102">
-        <f>B102-1</f>
+        <f t="shared" si="3"/>
         <v>99</v>
       </c>
       <c r="B102">
@@ -5824,9 +5841,9 @@
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103">
-        <f>B103-1</f>
+        <f t="shared" si="3"/>
         <v>100</v>
       </c>
       <c r="B103">
@@ -5845,9 +5862,9 @@
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104">
-        <f>B104-1</f>
+        <f t="shared" si="3"/>
         <v>101</v>
       </c>
       <c r="B104">
@@ -5866,9 +5883,9 @@
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105">
-        <f>B105-1</f>
+        <f t="shared" si="3"/>
         <v>102</v>
       </c>
       <c r="B105">
@@ -5887,9 +5904,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106">
-        <f>B106-1</f>
+        <f t="shared" si="3"/>
         <v>103</v>
       </c>
       <c r="B106">
@@ -5908,9 +5925,9 @@
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107">
-        <f>B107-1</f>
+        <f t="shared" si="3"/>
         <v>104</v>
       </c>
       <c r="B107">
@@ -5929,9 +5946,9 @@
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108">
-        <f>B108-1</f>
+        <f t="shared" si="3"/>
         <v>105</v>
       </c>
       <c r="B108">
@@ -5950,9 +5967,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109">
-        <f>B109-1</f>
+        <f t="shared" si="3"/>
         <v>106</v>
       </c>
       <c r="B109">
@@ -5971,9 +5988,9 @@
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110">
-        <f>B110-1</f>
+        <f t="shared" ref="A110:A141" si="4">B110-1</f>
         <v>107</v>
       </c>
       <c r="B110">
@@ -5992,9 +6009,9 @@
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111">
-        <f>B111-1</f>
+        <f t="shared" si="4"/>
         <v>108</v>
       </c>
       <c r="B111">
@@ -6013,9 +6030,9 @@
         <v>110</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112">
-        <f>B112-1</f>
+        <f t="shared" si="4"/>
         <v>109</v>
       </c>
       <c r="B112">
@@ -6034,9 +6051,9 @@
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113">
-        <f>B113-1</f>
+        <f t="shared" si="4"/>
         <v>110</v>
       </c>
       <c r="B113">
@@ -6055,9 +6072,9 @@
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114">
-        <f>B114-1</f>
+        <f t="shared" si="4"/>
         <v>111</v>
       </c>
       <c r="B114">
@@ -6076,9 +6093,9 @@
         <v>113</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115">
-        <f>B115-1</f>
+        <f t="shared" si="4"/>
         <v>112</v>
       </c>
       <c r="B115">
@@ -6097,9 +6114,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116">
-        <f>B116-1</f>
+        <f t="shared" si="4"/>
         <v>113</v>
       </c>
       <c r="B116">
@@ -6118,9 +6135,9 @@
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117">
-        <f>B117-1</f>
+        <f t="shared" si="4"/>
         <v>114</v>
       </c>
       <c r="B117">
@@ -6139,9 +6156,9 @@
         <v>116</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118">
-        <f>B118-1</f>
+        <f t="shared" si="4"/>
         <v>115</v>
       </c>
       <c r="B118">
@@ -6160,9 +6177,9 @@
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119">
-        <f>B119-1</f>
+        <f t="shared" si="4"/>
         <v>116</v>
       </c>
       <c r="B119">
@@ -6181,9 +6198,9 @@
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120">
-        <f>B120-1</f>
+        <f t="shared" si="4"/>
         <v>117</v>
       </c>
       <c r="B120">
@@ -6202,9 +6219,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121">
-        <f>B121-1</f>
+        <f t="shared" si="4"/>
         <v>118</v>
       </c>
       <c r="B121">
@@ -6223,9 +6240,9 @@
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122">
-        <f>B122-1</f>
+        <f t="shared" si="4"/>
         <v>119</v>
       </c>
       <c r="B122">
@@ -6244,9 +6261,9 @@
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123">
-        <f>B123-1</f>
+        <f t="shared" si="4"/>
         <v>120</v>
       </c>
       <c r="B123">
@@ -6265,9 +6282,9 @@
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124">
-        <f>B124-1</f>
+        <f t="shared" si="4"/>
         <v>121</v>
       </c>
       <c r="B124">
@@ -6286,9 +6303,9 @@
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125">
-        <f>B125-1</f>
+        <f t="shared" si="4"/>
         <v>122</v>
       </c>
       <c r="B125">
@@ -6307,9 +6324,9 @@
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126">
-        <f>B126-1</f>
+        <f t="shared" si="4"/>
         <v>123</v>
       </c>
       <c r="B126">
@@ -6328,9 +6345,9 @@
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127">
-        <f>B127-1</f>
+        <f t="shared" si="4"/>
         <v>124</v>
       </c>
       <c r="B127">
@@ -6349,9 +6366,9 @@
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128">
-        <f>B128-1</f>
+        <f t="shared" si="4"/>
         <v>125</v>
       </c>
       <c r="B128">
@@ -6370,9 +6387,9 @@
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129">
-        <f>B129-1</f>
+        <f t="shared" si="4"/>
         <v>126</v>
       </c>
       <c r="B129">
@@ -6391,9 +6408,9 @@
         <v>128</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130">
-        <f>B130-1</f>
+        <f t="shared" si="4"/>
         <v>127</v>
       </c>
       <c r="B130">
@@ -6412,9 +6429,9 @@
         <v>129</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131">
-        <f>B131-1</f>
+        <f t="shared" si="4"/>
         <v>128</v>
       </c>
       <c r="B131">
@@ -6433,9 +6450,9 @@
         <v>130</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132">
-        <f>B132-1</f>
+        <f t="shared" si="4"/>
         <v>129</v>
       </c>
       <c r="B132">
@@ -6454,9 +6471,9 @@
         <v>131</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133">
-        <f>B133-1</f>
+        <f t="shared" si="4"/>
         <v>130</v>
       </c>
       <c r="B133">
@@ -6475,9 +6492,9 @@
         <v>132</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134">
-        <f>B134-1</f>
+        <f t="shared" si="4"/>
         <v>131</v>
       </c>
       <c r="B134">
@@ -6496,9 +6513,9 @@
         <v>133</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135">
-        <f>B135-1</f>
+        <f t="shared" si="4"/>
         <v>132</v>
       </c>
       <c r="B135">
@@ -6517,9 +6534,9 @@
         <v>134</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136">
-        <f>B136-1</f>
+        <f t="shared" si="4"/>
         <v>133</v>
       </c>
       <c r="B136">
@@ -6538,9 +6555,9 @@
         <v>135</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137">
-        <f>B137-1</f>
+        <f t="shared" si="4"/>
         <v>134</v>
       </c>
       <c r="B137">
@@ -6559,9 +6576,9 @@
         <v>136</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138">
-        <f>B138-1</f>
+        <f t="shared" si="4"/>
         <v>135</v>
       </c>
       <c r="B138">
@@ -6580,9 +6597,9 @@
         <v>137</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139">
-        <f>B139-1</f>
+        <f t="shared" si="4"/>
         <v>136</v>
       </c>
       <c r="B139">
@@ -6601,9 +6618,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140">
-        <f>B140-1</f>
+        <f t="shared" si="4"/>
         <v>137</v>
       </c>
       <c r="B140">
@@ -6622,9 +6639,9 @@
         <v>139</v>
       </c>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141">
-        <f>B141-1</f>
+        <f t="shared" si="4"/>
         <v>138</v>
       </c>
       <c r="B141">
@@ -6643,9 +6660,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142">
-        <f>B142-1</f>
+        <f t="shared" ref="A142:A173" si="5">B142-1</f>
         <v>139</v>
       </c>
       <c r="B142">
@@ -6664,9 +6681,9 @@
         <v>141</v>
       </c>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143">
-        <f>B143-1</f>
+        <f t="shared" si="5"/>
         <v>140</v>
       </c>
       <c r="B143">
@@ -6685,9 +6702,9 @@
         <v>142</v>
       </c>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144">
-        <f>B144-1</f>
+        <f t="shared" si="5"/>
         <v>141</v>
       </c>
       <c r="B144">
@@ -6706,9 +6723,9 @@
         <v>143</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145">
-        <f>B145-1</f>
+        <f t="shared" si="5"/>
         <v>142</v>
       </c>
       <c r="B145">
@@ -6727,9 +6744,9 @@
         <v>144</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146">
-        <f>B146-1</f>
+        <f t="shared" si="5"/>
         <v>143</v>
       </c>
       <c r="B146">
@@ -6748,9 +6765,9 @@
         <v>145</v>
       </c>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147">
-        <f>B147-1</f>
+        <f t="shared" si="5"/>
         <v>144</v>
       </c>
       <c r="B147">
@@ -6769,9 +6786,9 @@
         <v>146</v>
       </c>
     </row>
-    <row r="148" spans="1:6">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148">
-        <f>B148-1</f>
+        <f t="shared" si="5"/>
         <v>145</v>
       </c>
       <c r="B148">
@@ -6790,9 +6807,9 @@
         <v>147</v>
       </c>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149">
-        <f>B149-1</f>
+        <f t="shared" si="5"/>
         <v>146</v>
       </c>
       <c r="B149">
@@ -6811,9 +6828,9 @@
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="1:6">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150">
-        <f>B150-1</f>
+        <f t="shared" si="5"/>
         <v>147</v>
       </c>
       <c r="B150">
@@ -6832,9 +6849,9 @@
         <v>149</v>
       </c>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151">
-        <f>B151-1</f>
+        <f t="shared" si="5"/>
         <v>148</v>
       </c>
       <c r="B151">
@@ -6853,9 +6870,9 @@
         <v>150</v>
       </c>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152">
-        <f>B152-1</f>
+        <f t="shared" si="5"/>
         <v>149</v>
       </c>
       <c r="B152">
@@ -6874,9 +6891,9 @@
         <v>151</v>
       </c>
     </row>
-    <row r="153" spans="1:6">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153">
-        <f>B153-1</f>
+        <f t="shared" si="5"/>
         <v>150</v>
       </c>
       <c r="B153">
@@ -6895,9 +6912,9 @@
         <v>152</v>
       </c>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154">
-        <f>B154-1</f>
+        <f t="shared" si="5"/>
         <v>151</v>
       </c>
       <c r="B154">
@@ -6916,9 +6933,9 @@
         <v>153</v>
       </c>
     </row>
-    <row r="155" spans="1:6">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155">
-        <f>B155-1</f>
+        <f t="shared" si="5"/>
         <v>152</v>
       </c>
       <c r="B155">
@@ -6937,9 +6954,9 @@
         <v>154</v>
       </c>
     </row>
-    <row r="156" spans="1:6">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156">
-        <f>B156-1</f>
+        <f t="shared" si="5"/>
         <v>153</v>
       </c>
       <c r="B156">
@@ -6958,9 +6975,9 @@
         <v>155</v>
       </c>
     </row>
-    <row r="157" spans="1:6">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157">
-        <f>B157-1</f>
+        <f t="shared" si="5"/>
         <v>154</v>
       </c>
       <c r="B157">
@@ -6979,9 +6996,9 @@
         <v>156</v>
       </c>
     </row>
-    <row r="158" spans="1:6">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158">
-        <f>B158-1</f>
+        <f t="shared" si="5"/>
         <v>155</v>
       </c>
       <c r="B158">
@@ -7000,9 +7017,9 @@
         <v>157</v>
       </c>
     </row>
-    <row r="159" spans="1:6">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159">
-        <f>B159-1</f>
+        <f t="shared" si="5"/>
         <v>156</v>
       </c>
       <c r="B159">
@@ -7021,9 +7038,9 @@
         <v>158</v>
       </c>
     </row>
-    <row r="160" spans="1:6">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160">
-        <f>B160-1</f>
+        <f t="shared" si="5"/>
         <v>157</v>
       </c>
       <c r="B160">
@@ -7042,9 +7059,9 @@
         <v>159</v>
       </c>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161">
-        <f>B161-1</f>
+        <f t="shared" si="5"/>
         <v>158</v>
       </c>
       <c r="B161">
@@ -7063,9 +7080,9 @@
         <v>160</v>
       </c>
     </row>
-    <row r="162" spans="1:6">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162">
-        <f>B162-1</f>
+        <f t="shared" si="5"/>
         <v>159</v>
       </c>
       <c r="B162">
@@ -7084,9 +7101,9 @@
         <v>161</v>
       </c>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163">
-        <f>B163-1</f>
+        <f t="shared" si="5"/>
         <v>160</v>
       </c>
       <c r="B163">
@@ -7105,9 +7122,9 @@
         <v>162</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164">
-        <f>B164-1</f>
+        <f t="shared" si="5"/>
         <v>161</v>
       </c>
       <c r="B164">
@@ -7126,31 +7143,53 @@
         <v>163</v>
       </c>
     </row>
-    <row r="165" spans="1:6">
-      <c r="B165">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D165" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="E165" t="s">
+        <v>333</v>
+      </c>
+      <c r="F165">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D166" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E166" t="s">
+        <v>333</v>
+      </c>
+      <c r="F166">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B167">
         <v>4</v>
       </c>
-      <c r="C165" t="s">
+      <c r="C167" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
-      <c r="B166">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B168">
         <v>23</v>
       </c>
-      <c r="C166" t="s">
+      <c r="C168" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
-      <c r="B167">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B169">
         <v>36</v>
       </c>
-      <c r="C167" t="s">
+      <c r="C169" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="181" spans="1:163">
+    <row r="181" spans="1:163" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>2</v>
       </c>
@@ -7647,10 +7686,5 @@
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
</xml_diff>